<commit_message>
chore(block-04): regenerate case_to_policy_mapping.xlsx after block-01/02 data fix
</commit_message>
<xml_diff>
--- a/data/block-04-risk-grading-policy/case_to_policy_mapping.xlsx
+++ b/data/block-04-risk-grading-policy/case_to_policy_mapping.xlsx
@@ -3562,7 +3562,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理</t>
@@ -3615,7 +3619,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -3668,7 +3676,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理</t>
@@ -3721,7 +3733,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -3774,7 +3790,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -3827,7 +3847,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
           <t>政务办公文件与邮件处理场景</t>
@@ -3880,7 +3904,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr"/>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -3933,7 +3961,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>政务通知短信批量发送场景</t>
@@ -3986,7 +4018,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr"/>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>gov-document-assistant</t>
+        </is>
+      </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
           <t>政务办公文件共享场景</t>
@@ -4039,7 +4075,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>gov-document-assistant</t>
+        </is>
+      </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
           <t>政务办公文件共享场景</t>
@@ -4092,7 +4132,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -4145,7 +4189,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
           <t>辖区商户服务短信发送管理</t>
@@ -4198,7 +4246,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr"/>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
           <t>其他</t>
@@ -4251,7 +4303,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr"/>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
           <t>政务办公场所门禁权限管理</t>
@@ -4304,7 +4360,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr"/>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
           <t>政务知识库检索场景</t>
@@ -4357,7 +4417,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr"/>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件检索场景</t>
@@ -4410,7 +4474,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr"/>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -4463,7 +4531,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -4516,7 +4588,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件系统</t>
@@ -4569,7 +4645,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -4622,7 +4702,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr"/>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
           <t>政务办公知识库检索场景</t>
@@ -4675,7 +4759,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
           <t>政务办公知识库检索场景</t>
@@ -4728,7 +4816,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr"/>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
           <t>政务办公场所门禁管理场景</t>
@@ -4781,7 +4873,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr"/>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>gov-calendar-task-assistant</t>
+        </is>
+      </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
           <t>政务会议日程管理</t>
@@ -4834,7 +4930,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr"/>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>gov-calendar-task-assistant</t>
+        </is>
+      </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
           <t>政务任务管理系统</t>
@@ -4887,7 +4987,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr"/>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
           <t>政务办公消息与邮件处理场景</t>
@@ -4940,7 +5044,11 @@
           <t>block-01</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr"/>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
           <t>政务办公浏览器使用场景</t>
@@ -4993,7 +5101,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr"/>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理</t>
@@ -5046,7 +5158,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C83" s="3" t="inlineStr"/>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -5099,7 +5215,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr"/>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理</t>
@@ -5152,7 +5272,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr"/>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -5205,7 +5329,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr"/>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -5258,7 +5386,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr"/>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
           <t>政务办公文件与邮件处理场景</t>
@@ -5311,7 +5443,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr"/>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -5364,7 +5500,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C89" s="3" t="inlineStr"/>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
           <t>政务通知短信批量发送场景</t>
@@ -5417,7 +5557,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr"/>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>gov-document-assistant</t>
+        </is>
+      </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
           <t>政务办公文件共享场景</t>
@@ -5470,7 +5614,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C91" s="3" t="inlineStr"/>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>gov-document-assistant</t>
+        </is>
+      </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
           <t>政务办公文件共享场景</t>
@@ -5523,7 +5671,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C92" s="3" t="inlineStr"/>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件处理场景</t>
@@ -5576,7 +5728,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr"/>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
           <t>辖区商户服务短信发送管理</t>
@@ -5629,7 +5785,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C94" s="3" t="inlineStr"/>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
           <t>其他</t>
@@ -5682,7 +5842,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C95" s="3" t="inlineStr"/>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
           <t>政务办公场所门禁权限管理</t>
@@ -5735,7 +5899,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr"/>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
           <t>政务知识库检索场景</t>
@@ -5788,7 +5956,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C97" s="3" t="inlineStr"/>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件检索场景</t>
@@ -5841,7 +6013,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C98" s="3" t="inlineStr"/>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -5894,7 +6070,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr"/>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -5947,7 +6127,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C100" s="3" t="inlineStr"/>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
           <t>政务办公邮件系统</t>
@@ -6000,7 +6184,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C101" s="3" t="inlineStr"/>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
           <t>政务邮件处理场景</t>
@@ -6053,7 +6241,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr"/>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
           <t>政务办公知识库检索场景</t>
@@ -6106,7 +6298,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr"/>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
           <t>政务办公知识库检索场景</t>
@@ -6159,7 +6355,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C104" s="3" t="inlineStr"/>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
           <t>政务办公场所门禁管理场景</t>
@@ -6212,7 +6412,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C105" s="3" t="inlineStr"/>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>gov-calendar-task-assistant</t>
+        </is>
+      </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
           <t>政务会议日程管理</t>
@@ -6265,7 +6469,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C106" s="3" t="inlineStr"/>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>gov-calendar-task-assistant</t>
+        </is>
+      </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
           <t>政务任务管理系统</t>
@@ -6318,7 +6526,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C107" s="3" t="inlineStr"/>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>gov-mail-assistant</t>
+        </is>
+      </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
           <t>政务办公消息与邮件处理场景</t>
@@ -6371,7 +6583,11 @@
           <t>block-02</t>
         </is>
       </c>
-      <c r="C108" s="3" t="inlineStr"/>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>gov-cross-department-assistant</t>
+        </is>
+      </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
           <t>政务办公浏览器使用场景</t>

</xml_diff>